<commit_message>
Rename app from "ICC Profile Validator" to "ICC Profile Tool"
The tool does more than validate — header browse, tag describe, XML/JSON
round-trip editing — so "Tool" reflects the scope better. Updated heading,
footer, page title, MANUAL.md, help-page generator, and all 12 locale
strings. Translation xlsx files and help.html regenerated.
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -493,10 +493,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ICC Profile Validator</v>
+        <v>ICC Profile Tool</v>
       </c>
       <c r="B12" t="str">
-        <v>ICC-Profilvalidator</v>
+        <v>ICC-Profil-Tool</v>
       </c>
     </row>
     <row r="13">
@@ -629,10 +629,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ICC Profile Validator · powered by IccProfLib</v>
+        <v>ICC Profile Tool · powered by IccProfLib</v>
       </c>
       <c r="B29" t="str">
-        <v>ICC-Profilvalidator · betrieben mit IccProfLib</v>
+        <v>ICC-Profil-Tool · betrieben mit IccProfLib</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
1.1.2: sync to merged iccDEV + localize validation status line
- WASM rebuilt from merged upstream iccDEV master (PR #1216, squashed as
  6a650e5), which includes the review-feedback refinements (CheckTagLayout
  frontier tracking, padding scan bounded to <=3-byte gaps, size_t range guard).
  Only iccprofiledump.wasm changes; the XML/JSON converters are byte-identical.
- Localize the validation status line: the wrapper's fixed status strings
  ("Profile is valid/non-compliant/...") and the best-effort/partial status now
  map to i18n keys (6 keys across all 12 locales). Validation message *bodies*
  remain in IccProfLib's source form (English) by design. Translations
  regenerated.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B81"/>
+  <dimension ref="A1:B87"/>
   <cols>
     <col min="1" max="1" width="50.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
@@ -845,215 +845,263 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>No warnings or errors found.</v>
+        <v>Profile is valid</v>
       </c>
       <c r="B56" t="str">
-        <v>Keine Warnungen oder Fehler gefunden.</v>
+        <v>Profil ist gültig</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Valid</v>
+        <v>Profile has warning(s)</v>
       </c>
       <c r="B57" t="str">
-        <v>Gültig</v>
+        <v>Profil hat Warnung(en)</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Warning</v>
+        <v>Profile is non-compliant</v>
       </c>
       <c r="B58" t="str">
-        <v>Warnung</v>
+        <v>Profil ist nicht konform</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Error</v>
+        <v>Critical validation error</v>
       </c>
       <c r="B59" t="str">
-        <v>Fehler</v>
+        <v>Kritischer Validierungsfehler</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Unknown</v>
+        <v>Unknown validation status</v>
       </c>
       <c r="B60" t="str">
-        <v>Unbekannt</v>
+        <v>Unbekannter Validierungsstatus</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>View in context</v>
+        <v>Critical — shown for inspection only</v>
       </c>
       <c r="B61" t="str">
-        <v>Im Kontext anzeigen</v>
+        <v>Kritisch — nur zur Ansicht angezeigt</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Validation detail</v>
+        <v>No warnings or errors found.</v>
       </c>
       <c r="B62" t="str">
-        <v>Validierungsdetail</v>
+        <v>Keine Warnungen oder Fehler gefunden.</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Triggered by</v>
+        <v>Valid</v>
       </c>
       <c r="B63" t="str">
-        <v>Ausgelöst durch</v>
+        <v>Gültig</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Field</v>
+        <v>Warning</v>
       </c>
       <c r="B64" t="str">
-        <v>Feld</v>
+        <v>Warnung</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Current value</v>
+        <v>Error</v>
       </c>
       <c r="B65" t="str">
-        <v>Aktueller Wert</v>
+        <v>Fehler</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Required: 0</v>
+        <v>Unknown</v>
       </c>
       <c r="B66" t="str">
-        <v>Erforderlich: 0</v>
+        <v>Unbekannt</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Expected: {value}</v>
+        <v>View in context</v>
       </c>
       <c r="B67" t="str">
-        <v>Erwartet: {value}</v>
+        <v>Im Kontext anzeigen</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Invalid</v>
+        <v>Validation detail</v>
       </c>
       <c r="B68" t="str">
-        <v>Ungültig</v>
+        <v>Validierungsdetail</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>This finding couldn't be tied to a specific field.</v>
+        <v>Triggered by</v>
       </c>
       <c r="B69" t="str">
-        <v>Dieser Befund konnte keinem bestimmten Feld zugeordnet werden.</v>
+        <v>Ausgelöst durch</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Close</v>
+        <v>Field</v>
       </c>
       <c r="B70" t="str">
-        <v>Schließen</v>
+        <v>Feld</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Loading XML editor…</v>
+        <v>Current value</v>
       </c>
       <c r="B71" t="str">
-        <v>Lade XML-Editor…</v>
+        <v>Aktueller Wert</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Loading JSON editor…</v>
+        <v>Required: 0</v>
       </c>
       <c r="B72" t="str">
-        <v>Lade JSON-Editor…</v>
+        <v>Erforderlich: 0</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>You have unsaved XML edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+        <v>Expected: {value}</v>
       </c>
       <c r="B73" t="str">
-        <v>Sie haben nicht gespeicherte XML-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+        <v>Erwartet: {value}</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>You have unsaved JSON edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+        <v>Invalid</v>
       </c>
       <c r="B74" t="str">
-        <v>Sie haben nicht gespeicherte JSON-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+        <v>Ungültig</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>● unsaved XML edits</v>
+        <v>This finding couldn't be tied to a specific field.</v>
       </c>
       <c r="B75" t="str">
-        <v>● nicht gespeicherte XML-Änderungen</v>
+        <v>Dieser Befund konnte keinem bestimmten Feld zugeordnet werden.</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>● unsaved JSON edits</v>
+        <v>Close</v>
       </c>
       <c r="B76" t="str">
-        <v>● nicht gespeicherte JSON-Änderungen</v>
+        <v>Schließen</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Click &lt;em&gt;Convert to XML&lt;/em&gt; to generate an editable XML representation of this profile. The XML is produced by the same IccLibXML code path used by the upstream &lt;code&gt;IccToXml&lt;/code&gt; tool.</v>
+        <v>Loading XML editor…</v>
       </c>
       <c r="B77" t="str">
-        <v>Klicken Sie auf &lt;em&gt;In XML konvertieren&lt;/em&gt;, um eine bearbeitbare XML-Darstellung dieses Profils zu erzeugen. Das XML wird vom gleichen IccLibXML-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToXml&lt;/code&gt; verwendet.</v>
+        <v>Lade XML-Editor…</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Click &lt;em&gt;Convert to JSON&lt;/em&gt; to generate an editable JSON representation of this profile. The JSON is produced by the same IccLibJSON code path used by the upstream &lt;code&gt;IccToJson&lt;/code&gt; tool.</v>
+        <v>Loading JSON editor…</v>
       </c>
       <c r="B78" t="str">
-        <v>Klicken Sie auf &lt;em&gt;In JSON konvertieren&lt;/em&gt;, um eine bearbeitbare JSON-Darstellung dieses Profils zu erzeugen. Das JSON wird vom gleichen IccLibJSON-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToJson&lt;/code&gt; verwendet.</v>
+        <v>Lade JSON-Editor…</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>indent</v>
+        <v>You have unsaved XML edits. Overwrite them with a fresh conversion from the ICC profile?</v>
       </c>
       <c r="B79" t="str">
-        <v>Einrückung</v>
+        <v>Sie haben nicht gespeicherte XML-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>sort keys</v>
+        <v>You have unsaved JSON edits. Overwrite them with a fresh conversion from the ICC profile?</v>
       </c>
       <c r="B80" t="str">
-        <v>Schlüssel sortieren</v>
+        <v>Sie haben nicht gespeicherte JSON-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
+        <v>● unsaved XML edits</v>
+      </c>
+      <c r="B81" t="str">
+        <v>● nicht gespeicherte XML-Änderungen</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>● unsaved JSON edits</v>
+      </c>
+      <c r="B82" t="str">
+        <v>● nicht gespeicherte JSON-Änderungen</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>Click &lt;em&gt;Convert to XML&lt;/em&gt; to generate an editable XML representation of this profile. The XML is produced by the same IccLibXML code path used by the upstream &lt;code&gt;IccToXml&lt;/code&gt; tool.</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Klicken Sie auf &lt;em&gt;In XML konvertieren&lt;/em&gt;, um eine bearbeitbare XML-Darstellung dieses Profils zu erzeugen. Das XML wird vom gleichen IccLibXML-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToXml&lt;/code&gt; verwendet.</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>Click &lt;em&gt;Convert to JSON&lt;/em&gt; to generate an editable JSON representation of this profile. The JSON is produced by the same IccLibJSON code path used by the upstream &lt;code&gt;IccToJson&lt;/code&gt; tool.</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Klicken Sie auf &lt;em&gt;In JSON konvertieren&lt;/em&gt;, um eine bearbeitbare JSON-Darstellung dieses Profils zu erzeugen. Das JSON wird vom gleichen IccLibJSON-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToJson&lt;/code&gt; verwendet.</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>indent</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Einrückung</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>sort keys</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Schlüssel sortieren</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
         <v>Profile written from edits, but re-validation failed:</v>
       </c>
-      <c r="B81" t="str">
+      <c r="B87" t="str">
         <v>Profil aus Änderungen geschrieben, aber Neuvalidierung fehlgeschlagen:</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B81"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B87"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Document Profile Assessment WG tab + sync translation spreadsheets
Add a "Profile Assessment WG" section (§3.4) to the user manual covering the
report's Security/Conformance/Quality grouping, the six verdicts, and the
clickable verdict-filter pills; renumber the following views and regenerate
help.html.

Regenerate translations/Eng-*.xlsx from the i18n dictionary so they reflect
the renamed tab label and pick up keys that had drifted since the last sync.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B87"/>
+  <dimension ref="A1:B98"/>
   <cols>
     <col min="1" max="1" width="50.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
@@ -605,503 +605,591 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Raw Output</v>
+        <v>Profile Assessment WG</v>
       </c>
       <c r="B26" t="str">
-        <v>Rohausgabe</v>
+        <v>Profile Assessment WG</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>XML</v>
+        <v>Raw Output</v>
       </c>
       <c r="B27" t="str">
-        <v>XML</v>
+        <v>Rohausgabe</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>JSON</v>
+        <v>XML</v>
       </c>
       <c r="B28" t="str">
-        <v>JSON</v>
+        <v>XML</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ICC Profile Tool · powered by IccProfLib</v>
+        <v>JSON</v>
       </c>
       <c r="B29" t="str">
-        <v>ICC-Profil-Tool · betrieben mit IccProfLib</v>
+        <v>JSON</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Error:</v>
+        <v>Loading Profile Assessment WG report…</v>
       </c>
       <c r="B30" t="str">
-        <v>Fehler:</v>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Convert to XML</v>
+        <v>Running Profile Assessment WG checks…</v>
       </c>
       <c r="B31" t="str">
-        <v>In XML konvertieren</v>
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Convert to JSON</v>
+        <v>Profile Assessment WG Report</v>
       </c>
       <c r="B32" t="str">
-        <v>In JSON konvertieren</v>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Convert to ICC</v>
+        <v>Security</v>
       </c>
       <c r="B33" t="str">
-        <v>In ICC konvertieren</v>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Converting to XML…</v>
+        <v>Conformance</v>
       </c>
       <c r="B34" t="str">
-        <v>Konvertiere in XML…</v>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Converting to JSON…</v>
+        <v>Quality</v>
       </c>
       <c r="B35" t="str">
-        <v>Konvertiere in JSON…</v>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Converting to ICC…</v>
+        <v>REPORT</v>
       </c>
       <c r="B36" t="str">
-        <v>Konvertiere in ICC…</v>
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Load ICC profile</v>
+        <v>FAIL</v>
       </c>
       <c r="B37" t="str">
-        <v>ICC-Profil laden</v>
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Drop zone for ICC profile files</v>
+        <v>checks</v>
       </c>
       <c r="B38" t="str">
-        <v>Ablagebereich für ICC-Profil-Dateien</v>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Profile ID</v>
+        <v>Generated by iccPawgReport (iccDEV) · ICC Profile Assessment Working Group checklist.</v>
       </c>
       <c r="B39" t="str">
-        <v>Profil-ID</v>
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>No tags found.</v>
+        <v>ICC Profile Tool · powered by IccProfLib</v>
       </c>
       <c r="B40" t="str">
-        <v>Keine Tags gefunden.</v>
+        <v>ICC-Profil-Tool · betrieben mit IccProfLib</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Tag Name</v>
+        <v>Error:</v>
       </c>
       <c r="B41" t="str">
-        <v>Tag-Name</v>
+        <v>Fehler:</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ID</v>
+        <v>Convert to XML</v>
       </c>
       <c r="B42" t="str">
-        <v>ID</v>
+        <v>In XML konvertieren</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Offset</v>
+        <v>Convert to JSON</v>
       </c>
       <c r="B43" t="str">
-        <v>Offset</v>
+        <v>In JSON konvertieren</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Size</v>
+        <v>Convert to ICC</v>
       </c>
       <c r="B44" t="str">
-        <v>Größe</v>
+        <v>In ICC konvertieren</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Pad</v>
+        <v>Converting to XML…</v>
       </c>
       <c r="B45" t="str">
-        <v>Auffüllung</v>
+        <v>Konvertiere in XML…</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Bytes changed since load</v>
+        <v>Converting to JSON…</v>
       </c>
       <c r="B46" t="str">
-        <v>Bytes seit dem Laden geändert</v>
+        <v>Konvertiere in JSON…</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Type</v>
+        <v>Converting to ICC…</v>
       </c>
       <c r="B47" t="str">
-        <v>Typ</v>
+        <v>Konvertiere in ICC…</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Array of {type}</v>
+        <v>Load ICC profile</v>
       </c>
       <c r="B48" t="str">
-        <v>Array von {type}</v>
+        <v>ICC-Profil laden</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>(No content)</v>
+        <v>Drop zone for ICC profile files</v>
       </c>
       <c r="B49" t="str">
-        <v>(Kein Inhalt)</v>
+        <v>Ablagebereich für ICC-Profil-Dateien</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>bytes</v>
+        <v>Profile ID</v>
       </c>
       <c r="B50" t="str">
-        <v>Bytes</v>
+        <v>Profil-ID</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Loading full description…</v>
+        <v>No tags found.</v>
       </c>
       <c r="B51" t="str">
-        <v>Lade vollständige Beschreibung…</v>
+        <v>Keine Tags gefunden.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Could not load full description:</v>
+        <v>Tag Name</v>
       </c>
       <c r="B52" t="str">
-        <v>Vollständige Beschreibung konnte nicht geladen werden:</v>
+        <v>Tag-Name</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>This profile could not be fully parsed and must not be applied. The header and tag directory below are shown for inspection only.</v>
+        <v>ID</v>
       </c>
       <c r="B53" t="str">
-        <v>Dieses Profil konnte nicht vollständig gelesen werden und darf nicht angewendet werden. Der Header und das Tag-Verzeichnis unten dienen nur zur Ansicht.</v>
+        <v>ID</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Tag contents unavailable — the profile could not be fully parsed.</v>
+        <v>Offset</v>
       </c>
       <c r="B54" t="str">
-        <v>Tag-Inhalt nicht verfügbar — das Profil konnte nicht vollständig gelesen werden.</v>
+        <v>Offset</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>No validation output</v>
+        <v>Size</v>
       </c>
       <c r="B55" t="str">
-        <v>Keine Validierungsausgabe</v>
+        <v>Größe</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Profile is valid</v>
+        <v>Pad</v>
       </c>
       <c r="B56" t="str">
-        <v>Profil ist gültig</v>
+        <v>Auffüllung</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Profile has warning(s)</v>
+        <v>Bytes changed since load</v>
       </c>
       <c r="B57" t="str">
-        <v>Profil hat Warnung(en)</v>
+        <v>Bytes seit dem Laden geändert</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Profile is non-compliant</v>
+        <v>Type</v>
       </c>
       <c r="B58" t="str">
-        <v>Profil ist nicht konform</v>
+        <v>Typ</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Critical validation error</v>
+        <v>Array of {type}</v>
       </c>
       <c r="B59" t="str">
-        <v>Kritischer Validierungsfehler</v>
+        <v>Array von {type}</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Unknown validation status</v>
+        <v>(No content)</v>
       </c>
       <c r="B60" t="str">
-        <v>Unbekannter Validierungsstatus</v>
+        <v>(Kein Inhalt)</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Critical — shown for inspection only</v>
+        <v>bytes</v>
       </c>
       <c r="B61" t="str">
-        <v>Kritisch — nur zur Ansicht angezeigt</v>
+        <v>Bytes</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>No warnings or errors found.</v>
+        <v>Loading full description…</v>
       </c>
       <c r="B62" t="str">
-        <v>Keine Warnungen oder Fehler gefunden.</v>
+        <v>Lade vollständige Beschreibung…</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Valid</v>
+        <v>Could not load full description:</v>
       </c>
       <c r="B63" t="str">
-        <v>Gültig</v>
+        <v>Vollständige Beschreibung konnte nicht geladen werden:</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Warning</v>
+        <v>This profile could not be fully parsed and must not be applied. The header and tag directory below are shown for inspection only.</v>
       </c>
       <c r="B64" t="str">
-        <v>Warnung</v>
+        <v>Dieses Profil konnte nicht vollständig gelesen werden und darf nicht angewendet werden. Der Header und das Tag-Verzeichnis unten dienen nur zur Ansicht.</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Error</v>
+        <v>Tag contents unavailable — the profile could not be fully parsed.</v>
       </c>
       <c r="B65" t="str">
-        <v>Fehler</v>
+        <v>Tag-Inhalt nicht verfügbar — das Profil konnte nicht vollständig gelesen werden.</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Unknown</v>
+        <v>No validation output</v>
       </c>
       <c r="B66" t="str">
-        <v>Unbekannt</v>
+        <v>Keine Validierungsausgabe</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>View in context</v>
+        <v>Profile is valid</v>
       </c>
       <c r="B67" t="str">
-        <v>Im Kontext anzeigen</v>
+        <v>Profil ist gültig</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Validation detail</v>
+        <v>Profile has warning(s)</v>
       </c>
       <c r="B68" t="str">
-        <v>Validierungsdetail</v>
+        <v>Profil hat Warnung(en)</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Triggered by</v>
+        <v>Profile is non-compliant</v>
       </c>
       <c r="B69" t="str">
-        <v>Ausgelöst durch</v>
+        <v>Profil ist nicht konform</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Field</v>
+        <v>Critical validation error</v>
       </c>
       <c r="B70" t="str">
-        <v>Feld</v>
+        <v>Kritischer Validierungsfehler</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Current value</v>
+        <v>Unknown validation status</v>
       </c>
       <c r="B71" t="str">
-        <v>Aktueller Wert</v>
+        <v>Unbekannter Validierungsstatus</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Required: 0</v>
+        <v>Critical — shown for inspection only</v>
       </c>
       <c r="B72" t="str">
-        <v>Erforderlich: 0</v>
+        <v>Kritisch — nur zur Ansicht angezeigt</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Expected: {value}</v>
+        <v>No warnings or errors found.</v>
       </c>
       <c r="B73" t="str">
-        <v>Erwartet: {value}</v>
+        <v>Keine Warnungen oder Fehler gefunden.</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Invalid</v>
+        <v>Valid</v>
       </c>
       <c r="B74" t="str">
-        <v>Ungültig</v>
+        <v>Gültig</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>This finding couldn't be tied to a specific field.</v>
+        <v>Warning</v>
       </c>
       <c r="B75" t="str">
-        <v>Dieser Befund konnte keinem bestimmten Feld zugeordnet werden.</v>
+        <v>Warnung</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Close</v>
+        <v>Error</v>
       </c>
       <c r="B76" t="str">
-        <v>Schließen</v>
+        <v>Fehler</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Loading XML editor…</v>
+        <v>Unknown</v>
       </c>
       <c r="B77" t="str">
-        <v>Lade XML-Editor…</v>
+        <v>Unbekannt</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Loading JSON editor…</v>
+        <v>View in context</v>
       </c>
       <c r="B78" t="str">
-        <v>Lade JSON-Editor…</v>
+        <v>Im Kontext anzeigen</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>You have unsaved XML edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+        <v>Validation detail</v>
       </c>
       <c r="B79" t="str">
-        <v>Sie haben nicht gespeicherte XML-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+        <v>Validierungsdetail</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>You have unsaved JSON edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+        <v>Triggered by</v>
       </c>
       <c r="B80" t="str">
-        <v>Sie haben nicht gespeicherte JSON-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+        <v>Ausgelöst durch</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>● unsaved XML edits</v>
+        <v>Field</v>
       </c>
       <c r="B81" t="str">
-        <v>● nicht gespeicherte XML-Änderungen</v>
+        <v>Feld</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>● unsaved JSON edits</v>
+        <v>Current value</v>
       </c>
       <c r="B82" t="str">
-        <v>● nicht gespeicherte JSON-Änderungen</v>
+        <v>Aktueller Wert</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Click &lt;em&gt;Convert to XML&lt;/em&gt; to generate an editable XML representation of this profile. The XML is produced by the same IccLibXML code path used by the upstream &lt;code&gt;IccToXml&lt;/code&gt; tool.</v>
+        <v>Required: 0</v>
       </c>
       <c r="B83" t="str">
-        <v>Klicken Sie auf &lt;em&gt;In XML konvertieren&lt;/em&gt;, um eine bearbeitbare XML-Darstellung dieses Profils zu erzeugen. Das XML wird vom gleichen IccLibXML-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToXml&lt;/code&gt; verwendet.</v>
+        <v>Erforderlich: 0</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>Click &lt;em&gt;Convert to JSON&lt;/em&gt; to generate an editable JSON representation of this profile. The JSON is produced by the same IccLibJSON code path used by the upstream &lt;code&gt;IccToJson&lt;/code&gt; tool.</v>
+        <v>Expected: {value}</v>
       </c>
       <c r="B84" t="str">
-        <v>Klicken Sie auf &lt;em&gt;In JSON konvertieren&lt;/em&gt;, um eine bearbeitbare JSON-Darstellung dieses Profils zu erzeugen. Das JSON wird vom gleichen IccLibJSON-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToJson&lt;/code&gt; verwendet.</v>
+        <v>Erwartet: {value}</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>indent</v>
+        <v>Invalid</v>
       </c>
       <c r="B85" t="str">
-        <v>Einrückung</v>
+        <v>Ungültig</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>sort keys</v>
+        <v>This finding couldn't be tied to a specific field.</v>
       </c>
       <c r="B86" t="str">
-        <v>Schlüssel sortieren</v>
+        <v>Dieser Befund konnte keinem bestimmten Feld zugeordnet werden.</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
+        <v>Close</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Schließen</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>Loading XML editor…</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Lade XML-Editor…</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>Loading JSON editor…</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Lade JSON-Editor…</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>You have unsaved XML edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Sie haben nicht gespeicherte XML-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>You have unsaved JSON edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+      </c>
+      <c r="B91" t="str">
+        <v>Sie haben nicht gespeicherte JSON-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>● unsaved XML edits</v>
+      </c>
+      <c r="B92" t="str">
+        <v>● nicht gespeicherte XML-Änderungen</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>● unsaved JSON edits</v>
+      </c>
+      <c r="B93" t="str">
+        <v>● nicht gespeicherte JSON-Änderungen</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>Click &lt;em&gt;Convert to XML&lt;/em&gt; to generate an editable XML representation of this profile. The XML is produced by the same IccLibXML code path used by the upstream &lt;code&gt;IccToXml&lt;/code&gt; tool.</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Klicken Sie auf &lt;em&gt;In XML konvertieren&lt;/em&gt;, um eine bearbeitbare XML-Darstellung dieses Profils zu erzeugen. Das XML wird vom gleichen IccLibXML-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToXml&lt;/code&gt; verwendet.</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>Click &lt;em&gt;Convert to JSON&lt;/em&gt; to generate an editable JSON representation of this profile. The JSON is produced by the same IccLibJSON code path used by the upstream &lt;code&gt;IccToJson&lt;/code&gt; tool.</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Klicken Sie auf &lt;em&gt;In JSON konvertieren&lt;/em&gt;, um eine bearbeitbare JSON-Darstellung dieses Profils zu erzeugen. Das JSON wird vom gleichen IccLibJSON-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToJson&lt;/code&gt; verwendet.</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>indent</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Einrückung</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>sort keys</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Schlüssel sortieren</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
         <v>Profile written from edits, but re-validation failed:</v>
       </c>
-      <c r="B87" t="str">
+      <c r="B98" t="str">
         <v>Profil aus Änderungen geschrieben, aber Neuvalidierung fehlgeschlagen:</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B87"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B98"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
1.1.5: URL-fragment launch (#url=…&tab=…)
Add a hash-fragment launch mechanism alongside the existing chardata
postMessage hand-off:

  https://chardata.colourbill.com/profiletool#url=<profile>&tab=<alias>

- url=  fetches the ICC profile and feeds the bytes through the same path
  as a local file (acsp check, ValidateIccProfile, 256 MB cap, best-effort
  fallback). Fetched bytes only flow into the validator, never re-sent.
- tab=  resolves to a stable tab key via two case-insensitive alias schemes
  (lib/tabs.js): whitespace-stripped display names and short codes
  (HEADER/TAGS/VAL/PAWG/RAW/XML/JSON). Aliases stay stable across label
  renames so links keep working.

Widen CSP connect-src to https: so url= can fetch from any HTTPS host
(subject to that host's CORS); script-src is unchanged. Document the
mechanism in MANUAL §6 and sync translation spreadsheets.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B98"/>
+  <dimension ref="A1:B100"/>
   <cols>
     <col min="1" max="1" width="50.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
@@ -637,23 +637,23 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Loading Profile Assessment WG report…</v>
+        <v>Invalid profile URL:</v>
       </c>
       <c r="B30" t="str">
-        <v/>
+        <v>Ungültige Profil-URL:</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Running Profile Assessment WG checks…</v>
+        <v>Could not fetch the profile from</v>
       </c>
       <c r="B31" t="str">
-        <v/>
+        <v>Profil konnte nicht abgerufen werden von</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Profile Assessment WG Report</v>
+        <v>Loading Profile Assessment WG report…</v>
       </c>
       <c r="B32" t="str">
         <v/>
@@ -661,7 +661,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Security</v>
+        <v>Running Profile Assessment WG checks…</v>
       </c>
       <c r="B33" t="str">
         <v/>
@@ -669,7 +669,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Conformance</v>
+        <v>Profile Assessment WG Report</v>
       </c>
       <c r="B34" t="str">
         <v/>
@@ -677,7 +677,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Quality</v>
+        <v>Security</v>
       </c>
       <c r="B35" t="str">
         <v/>
@@ -685,7 +685,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>REPORT</v>
+        <v>Conformance</v>
       </c>
       <c r="B36" t="str">
         <v/>
@@ -693,7 +693,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>FAIL</v>
+        <v>Quality</v>
       </c>
       <c r="B37" t="str">
         <v/>
@@ -701,7 +701,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>checks</v>
+        <v>REPORT</v>
       </c>
       <c r="B38" t="str">
         <v/>
@@ -709,7 +709,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Generated by iccPawgReport (iccDEV) · ICC Profile Assessment Working Group checklist.</v>
+        <v>FAIL</v>
       </c>
       <c r="B39" t="str">
         <v/>
@@ -717,479 +717,495 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ICC Profile Tool · powered by IccProfLib</v>
+        <v>checks</v>
       </c>
       <c r="B40" t="str">
-        <v>ICC-Profil-Tool · betrieben mit IccProfLib</v>
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Error:</v>
+        <v>Generated by iccPawgReport (iccDEV) · ICC Profile Assessment Working Group checklist.</v>
       </c>
       <c r="B41" t="str">
-        <v>Fehler:</v>
+        <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Convert to XML</v>
+        <v>ICC Profile Tool · powered by IccProfLib</v>
       </c>
       <c r="B42" t="str">
-        <v>In XML konvertieren</v>
+        <v>ICC-Profil-Tool · betrieben mit IccProfLib</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Convert to JSON</v>
+        <v>Error:</v>
       </c>
       <c r="B43" t="str">
-        <v>In JSON konvertieren</v>
+        <v>Fehler:</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Convert to ICC</v>
+        <v>Convert to XML</v>
       </c>
       <c r="B44" t="str">
-        <v>In ICC konvertieren</v>
+        <v>In XML konvertieren</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Converting to XML…</v>
+        <v>Convert to JSON</v>
       </c>
       <c r="B45" t="str">
-        <v>Konvertiere in XML…</v>
+        <v>In JSON konvertieren</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Converting to JSON…</v>
+        <v>Convert to ICC</v>
       </c>
       <c r="B46" t="str">
-        <v>Konvertiere in JSON…</v>
+        <v>In ICC konvertieren</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Converting to ICC…</v>
+        <v>Converting to XML…</v>
       </c>
       <c r="B47" t="str">
-        <v>Konvertiere in ICC…</v>
+        <v>Konvertiere in XML…</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Load ICC profile</v>
+        <v>Converting to JSON…</v>
       </c>
       <c r="B48" t="str">
-        <v>ICC-Profil laden</v>
+        <v>Konvertiere in JSON…</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Drop zone for ICC profile files</v>
+        <v>Converting to ICC…</v>
       </c>
       <c r="B49" t="str">
-        <v>Ablagebereich für ICC-Profil-Dateien</v>
+        <v>Konvertiere in ICC…</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Profile ID</v>
+        <v>Load ICC profile</v>
       </c>
       <c r="B50" t="str">
-        <v>Profil-ID</v>
+        <v>ICC-Profil laden</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>No tags found.</v>
+        <v>Drop zone for ICC profile files</v>
       </c>
       <c r="B51" t="str">
-        <v>Keine Tags gefunden.</v>
+        <v>Ablagebereich für ICC-Profil-Dateien</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Tag Name</v>
+        <v>Profile ID</v>
       </c>
       <c r="B52" t="str">
-        <v>Tag-Name</v>
+        <v>Profil-ID</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ID</v>
+        <v>No tags found.</v>
       </c>
       <c r="B53" t="str">
-        <v>ID</v>
+        <v>Keine Tags gefunden.</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Offset</v>
+        <v>Tag Name</v>
       </c>
       <c r="B54" t="str">
-        <v>Offset</v>
+        <v>Tag-Name</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Size</v>
+        <v>ID</v>
       </c>
       <c r="B55" t="str">
-        <v>Größe</v>
+        <v>ID</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Pad</v>
+        <v>Offset</v>
       </c>
       <c r="B56" t="str">
-        <v>Auffüllung</v>
+        <v>Offset</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Bytes changed since load</v>
+        <v>Size</v>
       </c>
       <c r="B57" t="str">
-        <v>Bytes seit dem Laden geändert</v>
+        <v>Größe</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Type</v>
+        <v>Pad</v>
       </c>
       <c r="B58" t="str">
-        <v>Typ</v>
+        <v>Auffüllung</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Array of {type}</v>
+        <v>Bytes changed since load</v>
       </c>
       <c r="B59" t="str">
-        <v>Array von {type}</v>
+        <v>Bytes seit dem Laden geändert</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>(No content)</v>
+        <v>Type</v>
       </c>
       <c r="B60" t="str">
-        <v>(Kein Inhalt)</v>
+        <v>Typ</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>bytes</v>
+        <v>Array of {type}</v>
       </c>
       <c r="B61" t="str">
-        <v>Bytes</v>
+        <v>Array von {type}</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Loading full description…</v>
+        <v>(No content)</v>
       </c>
       <c r="B62" t="str">
-        <v>Lade vollständige Beschreibung…</v>
+        <v>(Kein Inhalt)</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Could not load full description:</v>
+        <v>bytes</v>
       </c>
       <c r="B63" t="str">
-        <v>Vollständige Beschreibung konnte nicht geladen werden:</v>
+        <v>Bytes</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>This profile could not be fully parsed and must not be applied. The header and tag directory below are shown for inspection only.</v>
+        <v>Loading full description…</v>
       </c>
       <c r="B64" t="str">
-        <v>Dieses Profil konnte nicht vollständig gelesen werden und darf nicht angewendet werden. Der Header und das Tag-Verzeichnis unten dienen nur zur Ansicht.</v>
+        <v>Lade vollständige Beschreibung…</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Tag contents unavailable — the profile could not be fully parsed.</v>
+        <v>Could not load full description:</v>
       </c>
       <c r="B65" t="str">
-        <v>Tag-Inhalt nicht verfügbar — das Profil konnte nicht vollständig gelesen werden.</v>
+        <v>Vollständige Beschreibung konnte nicht geladen werden:</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>No validation output</v>
+        <v>This profile could not be fully parsed and must not be applied. The header and tag directory below are shown for inspection only.</v>
       </c>
       <c r="B66" t="str">
-        <v>Keine Validierungsausgabe</v>
+        <v>Dieses Profil konnte nicht vollständig gelesen werden und darf nicht angewendet werden. Der Header und das Tag-Verzeichnis unten dienen nur zur Ansicht.</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Profile is valid</v>
+        <v>Tag contents unavailable — the profile could not be fully parsed.</v>
       </c>
       <c r="B67" t="str">
-        <v>Profil ist gültig</v>
+        <v>Tag-Inhalt nicht verfügbar — das Profil konnte nicht vollständig gelesen werden.</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Profile has warning(s)</v>
+        <v>No validation output</v>
       </c>
       <c r="B68" t="str">
-        <v>Profil hat Warnung(en)</v>
+        <v>Keine Validierungsausgabe</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Profile is non-compliant</v>
+        <v>Profile is valid</v>
       </c>
       <c r="B69" t="str">
-        <v>Profil ist nicht konform</v>
+        <v>Profil ist gültig</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Critical validation error</v>
+        <v>Profile has warning(s)</v>
       </c>
       <c r="B70" t="str">
-        <v>Kritischer Validierungsfehler</v>
+        <v>Profil hat Warnung(en)</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Unknown validation status</v>
+        <v>Profile is non-compliant</v>
       </c>
       <c r="B71" t="str">
-        <v>Unbekannter Validierungsstatus</v>
+        <v>Profil ist nicht konform</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Critical — shown for inspection only</v>
+        <v>Critical validation error</v>
       </c>
       <c r="B72" t="str">
-        <v>Kritisch — nur zur Ansicht angezeigt</v>
+        <v>Kritischer Validierungsfehler</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>No warnings or errors found.</v>
+        <v>Unknown validation status</v>
       </c>
       <c r="B73" t="str">
-        <v>Keine Warnungen oder Fehler gefunden.</v>
+        <v>Unbekannter Validierungsstatus</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Valid</v>
+        <v>Critical — shown for inspection only</v>
       </c>
       <c r="B74" t="str">
-        <v>Gültig</v>
+        <v>Kritisch — nur zur Ansicht angezeigt</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Warning</v>
+        <v>No warnings or errors found.</v>
       </c>
       <c r="B75" t="str">
-        <v>Warnung</v>
+        <v>Keine Warnungen oder Fehler gefunden.</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Error</v>
+        <v>Valid</v>
       </c>
       <c r="B76" t="str">
-        <v>Fehler</v>
+        <v>Gültig</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Unknown</v>
+        <v>Warning</v>
       </c>
       <c r="B77" t="str">
-        <v>Unbekannt</v>
+        <v>Warnung</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>View in context</v>
+        <v>Error</v>
       </c>
       <c r="B78" t="str">
-        <v>Im Kontext anzeigen</v>
+        <v>Fehler</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Validation detail</v>
+        <v>Unknown</v>
       </c>
       <c r="B79" t="str">
-        <v>Validierungsdetail</v>
+        <v>Unbekannt</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Triggered by</v>
+        <v>View in context</v>
       </c>
       <c r="B80" t="str">
-        <v>Ausgelöst durch</v>
+        <v>Im Kontext anzeigen</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Field</v>
+        <v>Validation detail</v>
       </c>
       <c r="B81" t="str">
-        <v>Feld</v>
+        <v>Validierungsdetail</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Current value</v>
+        <v>Triggered by</v>
       </c>
       <c r="B82" t="str">
-        <v>Aktueller Wert</v>
+        <v>Ausgelöst durch</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Required: 0</v>
+        <v>Field</v>
       </c>
       <c r="B83" t="str">
-        <v>Erforderlich: 0</v>
+        <v>Feld</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>Expected: {value}</v>
+        <v>Current value</v>
       </c>
       <c r="B84" t="str">
-        <v>Erwartet: {value}</v>
+        <v>Aktueller Wert</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Invalid</v>
+        <v>Required: 0</v>
       </c>
       <c r="B85" t="str">
-        <v>Ungültig</v>
+        <v>Erforderlich: 0</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>This finding couldn't be tied to a specific field.</v>
+        <v>Expected: {value}</v>
       </c>
       <c r="B86" t="str">
-        <v>Dieser Befund konnte keinem bestimmten Feld zugeordnet werden.</v>
+        <v>Erwartet: {value}</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>Close</v>
+        <v>Invalid</v>
       </c>
       <c r="B87" t="str">
-        <v>Schließen</v>
+        <v>Ungültig</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Loading XML editor…</v>
+        <v>This finding couldn't be tied to a specific field.</v>
       </c>
       <c r="B88" t="str">
-        <v>Lade XML-Editor…</v>
+        <v>Dieser Befund konnte keinem bestimmten Feld zugeordnet werden.</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Loading JSON editor…</v>
+        <v>Close</v>
       </c>
       <c r="B89" t="str">
-        <v>Lade JSON-Editor…</v>
+        <v>Schließen</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>You have unsaved XML edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+        <v>Loading XML editor…</v>
       </c>
       <c r="B90" t="str">
-        <v>Sie haben nicht gespeicherte XML-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+        <v>Lade XML-Editor…</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>You have unsaved JSON edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+        <v>Loading JSON editor…</v>
       </c>
       <c r="B91" t="str">
-        <v>Sie haben nicht gespeicherte JSON-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+        <v>Lade JSON-Editor…</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>● unsaved XML edits</v>
+        <v>You have unsaved XML edits. Overwrite them with a fresh conversion from the ICC profile?</v>
       </c>
       <c r="B92" t="str">
-        <v>● nicht gespeicherte XML-Änderungen</v>
+        <v>Sie haben nicht gespeicherte XML-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>● unsaved JSON edits</v>
+        <v>You have unsaved JSON edits. Overwrite them with a fresh conversion from the ICC profile?</v>
       </c>
       <c r="B93" t="str">
-        <v>● nicht gespeicherte JSON-Änderungen</v>
+        <v>Sie haben nicht gespeicherte JSON-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>Click &lt;em&gt;Convert to XML&lt;/em&gt; to generate an editable XML representation of this profile. The XML is produced by the same IccLibXML code path used by the upstream &lt;code&gt;IccToXml&lt;/code&gt; tool.</v>
+        <v>● unsaved XML edits</v>
       </c>
       <c r="B94" t="str">
-        <v>Klicken Sie auf &lt;em&gt;In XML konvertieren&lt;/em&gt;, um eine bearbeitbare XML-Darstellung dieses Profils zu erzeugen. Das XML wird vom gleichen IccLibXML-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToXml&lt;/code&gt; verwendet.</v>
+        <v>● nicht gespeicherte XML-Änderungen</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>Click &lt;em&gt;Convert to JSON&lt;/em&gt; to generate an editable JSON representation of this profile. The JSON is produced by the same IccLibJSON code path used by the upstream &lt;code&gt;IccToJson&lt;/code&gt; tool.</v>
+        <v>● unsaved JSON edits</v>
       </c>
       <c r="B95" t="str">
-        <v>Klicken Sie auf &lt;em&gt;In JSON konvertieren&lt;/em&gt;, um eine bearbeitbare JSON-Darstellung dieses Profils zu erzeugen. Das JSON wird vom gleichen IccLibJSON-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToJson&lt;/code&gt; verwendet.</v>
+        <v>● nicht gespeicherte JSON-Änderungen</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>indent</v>
+        <v>Click &lt;em&gt;Convert to XML&lt;/em&gt; to generate an editable XML representation of this profile. The XML is produced by the same IccLibXML code path used by the upstream &lt;code&gt;IccToXml&lt;/code&gt; tool.</v>
       </c>
       <c r="B96" t="str">
-        <v>Einrückung</v>
+        <v>Klicken Sie auf &lt;em&gt;In XML konvertieren&lt;/em&gt;, um eine bearbeitbare XML-Darstellung dieses Profils zu erzeugen. Das XML wird vom gleichen IccLibXML-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToXml&lt;/code&gt; verwendet.</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>sort keys</v>
+        <v>Click &lt;em&gt;Convert to JSON&lt;/em&gt; to generate an editable JSON representation of this profile. The JSON is produced by the same IccLibJSON code path used by the upstream &lt;code&gt;IccToJson&lt;/code&gt; tool.</v>
       </c>
       <c r="B97" t="str">
-        <v>Schlüssel sortieren</v>
+        <v>Klicken Sie auf &lt;em&gt;In JSON konvertieren&lt;/em&gt;, um eine bearbeitbare JSON-Darstellung dieses Profils zu erzeugen. Das JSON wird vom gleichen IccLibJSON-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToJson&lt;/code&gt; verwendet.</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
+        <v>indent</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Einrückung</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>sort keys</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Schlüssel sortieren</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
         <v>Profile written from edits, but re-validation failed:</v>
       </c>
-      <c r="B98" t="str">
+      <c r="B100" t="str">
         <v>Profil aus Änderungen geschrieben, aber Neuvalidierung fehlgeschlagen:</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B98"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B100"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Harden #url= launch and analytics; remove innerHTML sinks
Security review fixes:

- analytics.js: pin GA page_location to origin+pathname, stripping the
  ?query/#fragment so the #url= profile target (and any token in it) is
  never shipped to Google Analytics.
- App.jsx: confirm before any cross-origin #url= fetch so a crafted link
  can't silently make the browser GET an arbitrary URL on load. Adds the
  url_confirm string to all 12 locales (+ regenerated translation xlsx).
- richText.jsx: render the XML/JSON converter placeholders' trusted
  i18n markup (<em>/<code>) as React nodes instead of via
  dangerouslySetInnerHTML, closing the latent XSS sink.
- CLAUDE.md: sync the security section with the live CSP and document the
  three new guards.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B131"/>
+  <dimension ref="A1:B132"/>
   <cols>
     <col min="1" max="1" width="50.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
@@ -885,575 +885,583 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Loading Profile Assessment WG report…</v>
+        <v>Load an ICC profile from this external site?</v>
       </c>
       <c r="B61" t="str">
-        <v>Profile-Assessment-WG-Bericht wird geladen…</v>
+        <v>Ein ICC-Profil von dieser externen Website laden?</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Running Profile Assessment WG checks…</v>
+        <v>Loading Profile Assessment WG report…</v>
       </c>
       <c r="B62" t="str">
-        <v>Profile-Assessment-WG-Prüfungen werden ausgeführt…</v>
+        <v>Profile-Assessment-WG-Bericht wird geladen…</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Profile Assessment WG Report</v>
+        <v>Running Profile Assessment WG checks…</v>
       </c>
       <c r="B63" t="str">
-        <v>Profile-Assessment-WG-Bericht</v>
+        <v>Profile-Assessment-WG-Prüfungen werden ausgeführt…</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Security</v>
+        <v>Profile Assessment WG Report</v>
       </c>
       <c r="B64" t="str">
-        <v>Sicherheit</v>
+        <v>Profile-Assessment-WG-Bericht</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Conformance</v>
+        <v>Security</v>
       </c>
       <c r="B65" t="str">
-        <v>Konformität</v>
+        <v>Sicherheit</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Quality</v>
+        <v>Conformance</v>
       </c>
       <c r="B66" t="str">
-        <v>Qualität</v>
+        <v>Konformität</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>REPORT</v>
+        <v>Quality</v>
       </c>
       <c r="B67" t="str">
-        <v>BERICHT</v>
+        <v>Qualität</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>FAIL</v>
+        <v>REPORT</v>
       </c>
       <c r="B68" t="str">
-        <v>FEHLGESCHLAGEN</v>
+        <v>BERICHT</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>checks</v>
+        <v>FAIL</v>
       </c>
       <c r="B69" t="str">
-        <v>Prüfungen</v>
+        <v>FEHLGESCHLAGEN</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Generated by iccPawgReport (iccDEV) · ICC Profile Assessment Working Group checklist.</v>
+        <v>checks</v>
       </c>
       <c r="B70" t="str">
-        <v>Erstellt von iccPawgReport (iccDEV) · Checkliste der ICC Profile Assessment Working Group.</v>
+        <v>Prüfungen</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>ICC Profile Tool · powered by IccProfLib</v>
+        <v>Generated by iccPawgReport (iccDEV) · ICC Profile Assessment Working Group checklist.</v>
       </c>
       <c r="B71" t="str">
-        <v>ICC-Profil-Tool · betrieben mit IccProfLib</v>
+        <v>Erstellt von iccPawgReport (iccDEV) · Checkliste der ICC Profile Assessment Working Group.</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Error:</v>
+        <v>ICC Profile Tool · powered by IccProfLib</v>
       </c>
       <c r="B72" t="str">
-        <v>Fehler:</v>
+        <v>ICC-Profil-Tool · betrieben mit IccProfLib</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Convert to XML</v>
+        <v>Error:</v>
       </c>
       <c r="B73" t="str">
-        <v>In XML konvertieren</v>
+        <v>Fehler:</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Convert to JSON</v>
+        <v>Convert to XML</v>
       </c>
       <c r="B74" t="str">
-        <v>In JSON konvertieren</v>
+        <v>In XML konvertieren</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Convert to ICC</v>
+        <v>Convert to JSON</v>
       </c>
       <c r="B75" t="str">
-        <v>In ICC konvertieren</v>
+        <v>In JSON konvertieren</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Converting to XML…</v>
+        <v>Convert to ICC</v>
       </c>
       <c r="B76" t="str">
-        <v>Konvertiere in XML…</v>
+        <v>In ICC konvertieren</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Converting to JSON…</v>
+        <v>Converting to XML…</v>
       </c>
       <c r="B77" t="str">
-        <v>Konvertiere in JSON…</v>
+        <v>Konvertiere in XML…</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Converting to ICC…</v>
+        <v>Converting to JSON…</v>
       </c>
       <c r="B78" t="str">
-        <v>Konvertiere in ICC…</v>
+        <v>Konvertiere in JSON…</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Load ICC profile</v>
+        <v>Converting to ICC…</v>
       </c>
       <c r="B79" t="str">
-        <v>ICC-Profil laden</v>
+        <v>Konvertiere in ICC…</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Drop zone for ICC profile files</v>
+        <v>Load ICC profile</v>
       </c>
       <c r="B80" t="str">
-        <v>Ablagebereich für ICC-Profil-Dateien</v>
+        <v>ICC-Profil laden</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Profile ID</v>
+        <v>Drop zone for ICC profile files</v>
       </c>
       <c r="B81" t="str">
-        <v>Profil-ID</v>
+        <v>Ablagebereich für ICC-Profil-Dateien</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>No tags found.</v>
+        <v>Profile ID</v>
       </c>
       <c r="B82" t="str">
-        <v>Keine Tags gefunden.</v>
+        <v>Profil-ID</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Tag Name</v>
+        <v>No tags found.</v>
       </c>
       <c r="B83" t="str">
-        <v>Tag-Name</v>
+        <v>Keine Tags gefunden.</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>ID</v>
+        <v>Tag Name</v>
       </c>
       <c r="B84" t="str">
-        <v>ID</v>
+        <v>Tag-Name</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Offset</v>
+        <v>ID</v>
       </c>
       <c r="B85" t="str">
-        <v>Offset</v>
+        <v>ID</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Size</v>
+        <v>Offset</v>
       </c>
       <c r="B86" t="str">
-        <v>Größe</v>
+        <v>Offset</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>Pad</v>
+        <v>Size</v>
       </c>
       <c r="B87" t="str">
-        <v>Auffüllung</v>
+        <v>Größe</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Bytes changed since load</v>
+        <v>Pad</v>
       </c>
       <c r="B88" t="str">
-        <v>Bytes seit dem Laden geändert</v>
+        <v>Auffüllung</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Type</v>
+        <v>Bytes changed since load</v>
       </c>
       <c r="B89" t="str">
-        <v>Typ</v>
+        <v>Bytes seit dem Laden geändert</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Array of {type}</v>
+        <v>Type</v>
       </c>
       <c r="B90" t="str">
-        <v>Array von {type}</v>
+        <v>Typ</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>(No content)</v>
+        <v>Array of {type}</v>
       </c>
       <c r="B91" t="str">
-        <v>(Kein Inhalt)</v>
+        <v>Array von {type}</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>bytes</v>
+        <v>(No content)</v>
       </c>
       <c r="B92" t="str">
-        <v>Bytes</v>
+        <v>(Kein Inhalt)</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>Loading full description…</v>
+        <v>bytes</v>
       </c>
       <c r="B93" t="str">
-        <v>Lade vollständige Beschreibung…</v>
+        <v>Bytes</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>Could not load full description:</v>
+        <v>Loading full description…</v>
       </c>
       <c r="B94" t="str">
-        <v>Vollständige Beschreibung konnte nicht geladen werden:</v>
+        <v>Lade vollständige Beschreibung…</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>This profile could not be fully parsed and must not be applied. The header and tag directory below are shown for inspection only.</v>
+        <v>Could not load full description:</v>
       </c>
       <c r="B95" t="str">
-        <v>Dieses Profil konnte nicht vollständig gelesen werden und darf nicht angewendet werden. Der Header und das Tag-Verzeichnis unten dienen nur zur Ansicht.</v>
+        <v>Vollständige Beschreibung konnte nicht geladen werden:</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Tag contents unavailable — the profile could not be fully parsed.</v>
+        <v>This profile could not be fully parsed and must not be applied. The header and tag directory below are shown for inspection only.</v>
       </c>
       <c r="B96" t="str">
-        <v>Tag-Inhalt nicht verfügbar — das Profil konnte nicht vollständig gelesen werden.</v>
+        <v>Dieses Profil konnte nicht vollständig gelesen werden und darf nicht angewendet werden. Der Header und das Tag-Verzeichnis unten dienen nur zur Ansicht.</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>No validation output</v>
+        <v>Tag contents unavailable — the profile could not be fully parsed.</v>
       </c>
       <c r="B97" t="str">
-        <v>Keine Validierungsausgabe</v>
+        <v>Tag-Inhalt nicht verfügbar — das Profil konnte nicht vollständig gelesen werden.</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>Profile is valid</v>
+        <v>No validation output</v>
       </c>
       <c r="B98" t="str">
-        <v>Profil ist gültig</v>
+        <v>Keine Validierungsausgabe</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Profile has warning(s)</v>
+        <v>Profile is valid</v>
       </c>
       <c r="B99" t="str">
-        <v>Profil hat Warnung(en)</v>
+        <v>Profil ist gültig</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>Profile is non-compliant</v>
+        <v>Profile has warning(s)</v>
       </c>
       <c r="B100" t="str">
-        <v>Profil ist nicht konform</v>
+        <v>Profil hat Warnung(en)</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Critical validation error</v>
+        <v>Profile is non-compliant</v>
       </c>
       <c r="B101" t="str">
-        <v>Kritischer Validierungsfehler</v>
+        <v>Profil ist nicht konform</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>Unknown validation status</v>
+        <v>Critical validation error</v>
       </c>
       <c r="B102" t="str">
-        <v>Unbekannter Validierungsstatus</v>
+        <v>Kritischer Validierungsfehler</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>Critical — shown for inspection only</v>
+        <v>Unknown validation status</v>
       </c>
       <c r="B103" t="str">
-        <v>Kritisch — nur zur Ansicht angezeigt</v>
+        <v>Unbekannter Validierungsstatus</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>No warnings or errors found.</v>
+        <v>Critical — shown for inspection only</v>
       </c>
       <c r="B104" t="str">
-        <v>Keine Warnungen oder Fehler gefunden.</v>
+        <v>Kritisch — nur zur Ansicht angezeigt</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>Valid</v>
+        <v>No warnings or errors found.</v>
       </c>
       <c r="B105" t="str">
-        <v>Gültig</v>
+        <v>Keine Warnungen oder Fehler gefunden.</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>Warning</v>
+        <v>Valid</v>
       </c>
       <c r="B106" t="str">
-        <v>Warnung</v>
+        <v>Gültig</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>Error</v>
+        <v>Warning</v>
       </c>
       <c r="B107" t="str">
-        <v>Fehler</v>
+        <v>Warnung</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>Unknown</v>
+        <v>Error</v>
       </c>
       <c r="B108" t="str">
-        <v>Unbekannt</v>
+        <v>Fehler</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>Pass</v>
+        <v>Unknown</v>
       </c>
       <c r="B109" t="str">
-        <v>Bestanden</v>
+        <v>Unbekannt</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>Fail</v>
+        <v>Pass</v>
       </c>
       <c r="B110" t="str">
-        <v>Fehlgeschlagen</v>
+        <v>Bestanden</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>View in context</v>
+        <v>Fail</v>
       </c>
       <c r="B111" t="str">
-        <v>Im Kontext anzeigen</v>
+        <v>Fehlgeschlagen</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>Validation detail</v>
+        <v>View in context</v>
       </c>
       <c r="B112" t="str">
-        <v>Validierungsdetail</v>
+        <v>Im Kontext anzeigen</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>Triggered by</v>
+        <v>Validation detail</v>
       </c>
       <c r="B113" t="str">
-        <v>Ausgelöst durch</v>
+        <v>Validierungsdetail</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>Field</v>
+        <v>Triggered by</v>
       </c>
       <c r="B114" t="str">
-        <v>Feld</v>
+        <v>Ausgelöst durch</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>Current value</v>
+        <v>Field</v>
       </c>
       <c r="B115" t="str">
-        <v>Aktueller Wert</v>
+        <v>Feld</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>Required: 0</v>
+        <v>Current value</v>
       </c>
       <c r="B116" t="str">
-        <v>Erforderlich: 0</v>
+        <v>Aktueller Wert</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>Expected: {value}</v>
+        <v>Required: 0</v>
       </c>
       <c r="B117" t="str">
-        <v>Erwartet: {value}</v>
+        <v>Erforderlich: 0</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>Invalid</v>
+        <v>Expected: {value}</v>
       </c>
       <c r="B118" t="str">
-        <v>Ungültig</v>
+        <v>Erwartet: {value}</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>This finding couldn't be tied to a specific field.</v>
+        <v>Invalid</v>
       </c>
       <c r="B119" t="str">
-        <v>Dieser Befund konnte keinem bestimmten Feld zugeordnet werden.</v>
+        <v>Ungültig</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>Close</v>
+        <v>This finding couldn't be tied to a specific field.</v>
       </c>
       <c r="B120" t="str">
-        <v>Schließen</v>
+        <v>Dieser Befund konnte keinem bestimmten Feld zugeordnet werden.</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>Loading XML editor…</v>
+        <v>Close</v>
       </c>
       <c r="B121" t="str">
-        <v>Lade XML-Editor…</v>
+        <v>Schließen</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>Loading JSON editor…</v>
+        <v>Loading XML editor…</v>
       </c>
       <c r="B122" t="str">
-        <v>Lade JSON-Editor…</v>
+        <v>Lade XML-Editor…</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>You have unsaved XML edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+        <v>Loading JSON editor…</v>
       </c>
       <c r="B123" t="str">
-        <v>Sie haben nicht gespeicherte XML-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+        <v>Lade JSON-Editor…</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>You have unsaved JSON edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+        <v>You have unsaved XML edits. Overwrite them with a fresh conversion from the ICC profile?</v>
       </c>
       <c r="B124" t="str">
-        <v>Sie haben nicht gespeicherte JSON-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+        <v>Sie haben nicht gespeicherte XML-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>● unsaved XML edits</v>
+        <v>You have unsaved JSON edits. Overwrite them with a fresh conversion from the ICC profile?</v>
       </c>
       <c r="B125" t="str">
-        <v>● nicht gespeicherte XML-Änderungen</v>
+        <v>Sie haben nicht gespeicherte JSON-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>● unsaved JSON edits</v>
+        <v>● unsaved XML edits</v>
       </c>
       <c r="B126" t="str">
-        <v>● nicht gespeicherte JSON-Änderungen</v>
+        <v>● nicht gespeicherte XML-Änderungen</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>Click &lt;em&gt;Convert to XML&lt;/em&gt; to generate an editable XML representation of this profile. The XML is produced by the same IccLibXML code path used by the upstream &lt;code&gt;IccToXml&lt;/code&gt; tool.</v>
+        <v>● unsaved JSON edits</v>
       </c>
       <c r="B127" t="str">
-        <v>Klicken Sie auf &lt;em&gt;In XML konvertieren&lt;/em&gt;, um eine bearbeitbare XML-Darstellung dieses Profils zu erzeugen. Das XML wird vom gleichen IccLibXML-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToXml&lt;/code&gt; verwendet.</v>
+        <v>● nicht gespeicherte JSON-Änderungen</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>Click &lt;em&gt;Convert to JSON&lt;/em&gt; to generate an editable JSON representation of this profile. The JSON is produced by the same IccLibJSON code path used by the upstream &lt;code&gt;IccToJson&lt;/code&gt; tool.</v>
+        <v>Click &lt;em&gt;Convert to XML&lt;/em&gt; to generate an editable XML representation of this profile. The XML is produced by the same IccLibXML code path used by the upstream &lt;code&gt;IccToXml&lt;/code&gt; tool.</v>
       </c>
       <c r="B128" t="str">
-        <v>Klicken Sie auf &lt;em&gt;In JSON konvertieren&lt;/em&gt;, um eine bearbeitbare JSON-Darstellung dieses Profils zu erzeugen. Das JSON wird vom gleichen IccLibJSON-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToJson&lt;/code&gt; verwendet.</v>
+        <v>Klicken Sie auf &lt;em&gt;In XML konvertieren&lt;/em&gt;, um eine bearbeitbare XML-Darstellung dieses Profils zu erzeugen. Das XML wird vom gleichen IccLibXML-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToXml&lt;/code&gt; verwendet.</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>indent</v>
+        <v>Click &lt;em&gt;Convert to JSON&lt;/em&gt; to generate an editable JSON representation of this profile. The JSON is produced by the same IccLibJSON code path used by the upstream &lt;code&gt;IccToJson&lt;/code&gt; tool.</v>
       </c>
       <c r="B129" t="str">
-        <v>Einrückung</v>
+        <v>Klicken Sie auf &lt;em&gt;In JSON konvertieren&lt;/em&gt;, um eine bearbeitbare JSON-Darstellung dieses Profils zu erzeugen. Das JSON wird vom gleichen IccLibJSON-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToJson&lt;/code&gt; verwendet.</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>sort keys</v>
+        <v>indent</v>
       </c>
       <c r="B130" t="str">
-        <v>Schlüssel sortieren</v>
+        <v>Einrückung</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
+        <v>sort keys</v>
+      </c>
+      <c r="B131" t="str">
+        <v>Schlüssel sortieren</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
         <v>Profile written from edits, but re-validation failed:</v>
       </c>
-      <c r="B131" t="str">
+      <c r="B132" t="str">
         <v>Profil aus Änderungen geschrieben, aber Neuvalidierung fehlgeschlagen:</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B131"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B132"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
1.8.1: localize Profile Statistics
1.8.1 — Profile Statistics: full localization

Translates the Profile Statistics strings — section heading, intro, the
Rendering intent / Gamut volume / Round-trip ΔE column labels, mean/P90/max, and
the Absolute Colorimetric intent name — into all 11 non-English languages, and
regenerates the translation spreadsheets from the i18n dictionary.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014NduGJdN1Sp1KPX3KSjMPn
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B190"/>
+  <dimension ref="A1:B200"/>
   <cols>
     <col min="1" max="1" width="50.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
@@ -797,330 +797,330 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Channels with many reversals show only the {shown} largest by ΔL*.</v>
+        <v>Absolute Colorimetric</v>
       </c>
       <c r="B50" t="str">
-        <v>Kanäle mit vielen Umkehrungen zeigen nur die {shown} größten nach ΔL*.</v>
+        <v>Absolut farbmetrisch</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Show more ({n})</v>
+        <v>Profile Statistics</v>
       </c>
       <c r="B51" t="str">
-        <v>Mehr anzeigen ({n})</v>
+        <v>Profilstatistik</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>All</v>
+        <v>Whole-profile metrics per rendering intent: the gamut volume enclosed by the device→PCS transform (ΔE*ab³), and the B2A round-trip accuracy — ΔE*ab of a Lab → device → Lab round trip through the profile.</v>
       </c>
       <c r="B52" t="str">
-        <v>Alle</v>
+        <v>Profilweite Kennzahlen je Render-Intent: das vom Gerät→PCS-Transform umschlossene Gamut-Volumen (ΔE*ab³) und die B2A-Roundtrip-Genauigkeit — ΔE*ab eines Lab → Gerät → Lab-Umlaufs durch das Profil.</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Analysing…</v>
+        <v>No device↔PCS CLUTs in this profile — profile statistics do not apply (e.g. a matrix/TRC display profile).</v>
       </c>
       <c r="B53" t="str">
-        <v>Analyse läuft…</v>
+        <v>Keine Gerät↔PCS-CLUTs in diesem Profil — die Profilstatistik ist nicht anwendbar (z. B. ein Matrix/TRC-Displayprofil).</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Analysis</v>
+        <v>Rendering intent</v>
       </c>
       <c r="B54" t="str">
-        <v>Analyse</v>
+        <v>Render-Intent</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Profile-wide quality analyses derived from the device-to-PCS transform.</v>
+        <v>Gamut volume (ΔE³)</v>
       </c>
       <c r="B55" t="str">
-        <v>Profilweite Qualitätsanalysen, abgeleitet aus der Gerät→PCS-Transformation.</v>
+        <v>Gamut-Volumen (ΔE³)</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>L* Tone Reversal</v>
+        <v>Round-trip ΔE</v>
       </c>
       <c r="B56" t="str">
-        <v>L*-Tonwertumkehr</v>
+        <v>Roundtrip-ΔE</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Adding ink should never make a colour lighter. Each device channel is swept while the others are held fixed; any step where L* rises is flagged. Algorithm originally due to Harold Boll.</v>
+        <v>mean</v>
       </c>
       <c r="B57" t="str">
-        <v>Mehr Farbe sollte eine Farbe nie heller machen. Jeder Gerätekanal wird durchlaufen, die anderen bleiben fest; jeder Schritt, in dem L* steigt, wird markiert. Algorithmus ursprünglich von Harold Boll.</v>
+        <v>Mittel</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>No device-to-PCS CLUT in this profile, so the L* reversal scan does not apply (for example, a matrix/TRC display profile).</v>
+        <v>P90</v>
       </c>
       <c r="B58" t="str">
-        <v>Keine Gerät→PCS-CLUT in diesem Profil – die L*-Umkehrprüfung ist nicht anwendbar (z. B. ein Matrix-/TRC-Anzeigeprofil).</v>
+        <v>P90</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>LUT table</v>
+        <v>max</v>
       </c>
       <c r="B59" t="str">
-        <v>LUT-Tabelle</v>
+        <v>Max.</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ΔL* threshold (ε)</v>
+        <v>Channels with many reversals show only the {shown} largest by ΔL*.</v>
       </c>
       <c r="B60" t="str">
-        <v>ΔL*-Schwelle (ε)</v>
+        <v>Kanäle mit vielen Umkehrungen zeigen nur die {shown} größten nach ΔL*.</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>{n} reversals above ε = {eps}</v>
+        <v>Show more ({n})</v>
       </c>
       <c r="B61" t="str">
-        <v>{n} Umkehrungen über ε = {eps}</v>
+        <v>Mehr anzeigen ({n})</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>No L* reversals above ε = {eps}</v>
+        <v>All</v>
       </c>
       <c r="B62" t="str">
-        <v>Keine L*-Umkehrungen über ε = {eps}</v>
+        <v>Alle</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Channel</v>
+        <v>Analysing…</v>
       </c>
       <c r="B63" t="str">
-        <v>Kanal</v>
+        <v>Analyse läuft…</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Ink (low → high)</v>
+        <v>Analysis</v>
       </c>
       <c r="B64" t="str">
-        <v>Farbe (niedrig → hoch)</v>
+        <v>Analyse</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Plot</v>
+        <v>Profile-wide quality analyses derived from the device-to-PCS transform.</v>
       </c>
       <c r="B65" t="str">
-        <v>Diagramm</v>
+        <v>Profilweite Qualitätsanalysen, abgeleitet aus der Gerät→PCS-Transformation.</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Raw Output</v>
+        <v>L* Tone Reversal</v>
       </c>
       <c r="B66" t="str">
-        <v>Rohausgabe</v>
+        <v>L*-Tonwertumkehr</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>XML</v>
+        <v>Adding ink should never make a colour lighter. Each device channel is swept while the others are held fixed; any step where L* rises is flagged. Algorithm originally due to Harold Boll.</v>
       </c>
       <c r="B67" t="str">
-        <v>XML</v>
+        <v>Mehr Farbe sollte eine Farbe nie heller machen. Jeder Gerätekanal wird durchlaufen, die anderen bleiben fest; jeder Schritt, in dem L* steigt, wird markiert. Algorithmus ursprünglich von Harold Boll.</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>JSON</v>
+        <v>No device-to-PCS CLUT in this profile, so the L* reversal scan does not apply (for example, a matrix/TRC display profile).</v>
       </c>
       <c r="B68" t="str">
-        <v>JSON</v>
+        <v>Keine Gerät→PCS-CLUT in diesem Profil – die L*-Umkehrprüfung ist nicht anwendbar (z. B. ein Matrix-/TRC-Anzeigeprofil).</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Curves</v>
+        <v>LUT table</v>
       </c>
       <c r="B69" t="str">
-        <v>Kurven</v>
+        <v>LUT-Tabelle</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Input curves</v>
+        <v>ΔL* threshold (ε)</v>
       </c>
       <c r="B70" t="str">
-        <v>Eingangskurven</v>
+        <v>ΔL*-Schwelle (ε)</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Output curves</v>
+        <v>{n} reversals above ε = {eps}</v>
       </c>
       <c r="B71" t="str">
-        <v>Ausgangskurven</v>
+        <v>{n} Umkehrungen über ε = {eps}</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>CLUT image</v>
+        <v>No L* reversals above ε = {eps}</v>
       </c>
       <c r="B72" t="str">
-        <v>CLUT-Bild</v>
+        <v>Keine L*-Umkehrungen über ε = {eps}</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Gamut image</v>
+        <v>Channel</v>
       </c>
       <c r="B73" t="str">
-        <v>Gamut-Bild</v>
+        <v>Kanal</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Chromaticity</v>
+        <v>Ink (low → high)</v>
       </c>
       <c r="B74" t="str">
-        <v>Chromazität</v>
+        <v>Farbe (niedrig → hoch)</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Scatter plot</v>
+        <v>Plot</v>
       </c>
       <c r="B75" t="str">
-        <v>Streudiagramm</v>
+        <v>Diagramm</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Tone response curve</v>
+        <v>Raw Output</v>
       </c>
       <c r="B76" t="str">
-        <v>Tonwertkurve</v>
+        <v>Rohausgabe</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Curve table</v>
+        <v>XML</v>
       </c>
       <c r="B77" t="str">
-        <v>Kurventabelle</v>
+        <v>XML</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Tables</v>
+        <v>JSON</v>
       </c>
       <c r="B78" t="str">
-        <v>Tabellen</v>
+        <v>JSON</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Data</v>
+        <v>Curves</v>
       </c>
       <c r="B79" t="str">
-        <v>Daten</v>
+        <v>Kurven</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Evaluate</v>
+        <v>Input curves</v>
       </c>
       <c r="B80" t="str">
-        <v>Auswerten</v>
+        <v>Eingangskurven</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Loading…</v>
+        <v>Output curves</v>
       </c>
       <c r="B81" t="str">
-        <v>Wird geladen…</v>
+        <v>Ausgangskurven</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Input</v>
+        <v>CLUT image</v>
       </c>
       <c r="B82" t="str">
-        <v>Eingang</v>
+        <v>CLUT-Bild</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Output</v>
+        <v>Gamut image</v>
       </c>
       <c r="B83" t="str">
-        <v>Ausgang</v>
+        <v>Gamut-Bild</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>Floating point</v>
+        <v>Chromaticity</v>
       </c>
       <c r="B84" t="str">
-        <v>Gleitkomma</v>
+        <v>Chromazität</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Grid point</v>
+        <v>Scatter plot</v>
       </c>
       <c r="B85" t="str">
-        <v>Gitterpunkt</v>
+        <v>Streudiagramm</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Normalized</v>
+        <v>Tone response curve</v>
       </c>
       <c r="B86" t="str">
-        <v>Normalisiert</v>
+        <v>Tonwertkurve</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>Human</v>
+        <v>Curve table</v>
       </c>
       <c r="B87" t="str">
-        <v>Lesbar</v>
+        <v>Kurventabelle</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Device → PCS</v>
+        <v>Tables</v>
       </c>
       <c r="B88" t="str">
-        <v>Gerät → PCS</v>
+        <v>Tabellen</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>PCS → Device</v>
+        <v>Data</v>
       </c>
       <c r="B89" t="str">
-        <v>PCS → Gerät</v>
+        <v>Daten</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>No CLUT grid</v>
+        <v>Evaluate</v>
       </c>
       <c r="B90" t="str">
-        <v>Kein CLUT-Gitter</v>
+        <v>Auswerten</v>
       </c>
     </row>
     <row r="91">
@@ -1133,799 +1133,879 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Neutral = in gamut · red = out of gamut</v>
+        <v>Input</v>
       </c>
       <c r="B92" t="str">
-        <v>Neutral = im Gamut · rot = außerhalb des Gamuts</v>
+        <v>Eingang</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>Invalid profile URL:</v>
+        <v>Output</v>
       </c>
       <c r="B93" t="str">
-        <v>Ungültige Profil-URL:</v>
+        <v>Ausgang</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>Could not fetch the profile from</v>
+        <v>Floating point</v>
       </c>
       <c r="B94" t="str">
-        <v>Profil konnte nicht abgerufen werden von</v>
+        <v>Gleitkomma</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>Load an ICC profile from this external site?</v>
+        <v>Grid point</v>
       </c>
       <c r="B95" t="str">
-        <v>Ein ICC-Profil von dieser externen Website laden?</v>
+        <v>Gitterpunkt</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Loading Profile Assessment WG report…</v>
+        <v>Normalized</v>
       </c>
       <c r="B96" t="str">
-        <v>Profile-Assessment-WG-Bericht wird geladen…</v>
+        <v>Normalisiert</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>Running Profile Assessment WG checks…</v>
+        <v>Human</v>
       </c>
       <c r="B97" t="str">
-        <v>Profile-Assessment-WG-Prüfungen werden ausgeführt…</v>
+        <v>Lesbar</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>Profile Assessment WG Report</v>
+        <v>Device → PCS</v>
       </c>
       <c r="B98" t="str">
-        <v>Profile-Assessment-WG-Bericht</v>
+        <v>Gerät → PCS</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Security</v>
+        <v>PCS → Device</v>
       </c>
       <c r="B99" t="str">
-        <v>Sicherheit</v>
+        <v>PCS → Gerät</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>Conformance</v>
+        <v>No CLUT grid</v>
       </c>
       <c r="B100" t="str">
-        <v>Konformität</v>
+        <v>Kein CLUT-Gitter</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Quality</v>
+        <v>Loading…</v>
       </c>
       <c r="B101" t="str">
-        <v>Qualität</v>
+        <v>Wird geladen…</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>REPORT</v>
+        <v>Neutral = in gamut · red = out of gamut</v>
       </c>
       <c r="B102" t="str">
-        <v>BERICHT</v>
+        <v>Neutral = im Gamut · rot = außerhalb des Gamuts</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>FAIL</v>
+        <v>Invalid profile URL:</v>
       </c>
       <c r="B103" t="str">
-        <v>FEHLGESCHLAGEN</v>
+        <v>Ungültige Profil-URL:</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>checks</v>
+        <v>Could not fetch the profile from</v>
       </c>
       <c r="B104" t="str">
-        <v>Prüfungen</v>
+        <v>Profil konnte nicht abgerufen werden von</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>Generated by iccPawgReport (iccDEV) · ICC Profile Assessment Working Group checklist.</v>
+        <v>Load an ICC profile from this external site?</v>
       </c>
       <c r="B105" t="str">
-        <v>Erstellt von iccPawgReport (iccDEV) · Checkliste der ICC Profile Assessment Working Group.</v>
+        <v>Ein ICC-Profil von dieser externen Website laden?</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>ICC Profile Tool · powered by IccProfLib</v>
+        <v>Loading Profile Assessment WG report…</v>
       </c>
       <c r="B106" t="str">
-        <v>ICC-Profil-Tool · betrieben mit IccProfLib</v>
+        <v>Profile-Assessment-WG-Bericht wird geladen…</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>ICC Profile Tool</v>
+        <v>Running Profile Assessment WG checks…</v>
       </c>
       <c r="B107" t="str">
-        <v>ICC-Profil-Tool</v>
+        <v>Profile-Assessment-WG-Prüfungen werden ausgeführt…</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>Powered by {lib}</v>
+        <v>Profile Assessment WG Report</v>
       </c>
       <c r="B108" t="str">
-        <v>Betrieben mit {lib}</v>
+        <v>Profile-Assessment-WG-Bericht</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>Subscribe</v>
+        <v>Security</v>
       </c>
       <c r="B109" t="str">
-        <v>Abonnieren</v>
+        <v>Sicherheit</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>Get notified about new profiletool releases</v>
+        <v>Conformance</v>
       </c>
       <c r="B110" t="str">
-        <v>Bei neuen profiletool-Releases benachrichtigt werden</v>
+        <v>Konformität</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>Get notified about new releases</v>
+        <v>Quality</v>
       </c>
       <c r="B111" t="str">
-        <v>Bei neuen Releases benachrichtigt werden</v>
+        <v>Qualität</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>Close</v>
+        <v>REPORT</v>
       </c>
       <c r="B112" t="str">
-        <v>Schließen</v>
+        <v>BERICHT</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>We’ll email you when a new major or minor profiletool release ships. Patch releases are skipped. Your address is reviewed manually before being added.</v>
+        <v>FAIL</v>
       </c>
       <c r="B113" t="str">
-        <v>Wir benachrichtigen Sie per E-Mail, sobald ein neues Major- oder Minor-Release von profiletool erscheint. Patch-Releases werden übersprungen. Ihre Adresse wird manuell geprüft, bevor sie aufgenommen wird.</v>
+        <v>FEHLGESCHLAGEN</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>Email address</v>
+        <v>checks</v>
       </c>
       <c r="B114" t="str">
-        <v>E-Mail-Adresse</v>
+        <v>Prüfungen</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>you@example.com</v>
+        <v>Generated by iccPawgReport (iccDEV) · ICC Profile Assessment Working Group checklist.</v>
       </c>
       <c r="B115" t="str">
-        <v>sie@example.com</v>
+        <v>Erstellt von iccPawgReport (iccDEV) · Checkliste der ICC Profile Assessment Working Group.</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>How will you use profiletool?</v>
+        <v>ICC Profile Tool · powered by IccProfLib</v>
       </c>
       <c r="B116" t="str">
-        <v>Wofür werden Sie profiletool nutzen?</v>
+        <v>ICC-Profil-Tool · betrieben mit IccProfLib</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>(optional)</v>
+        <v>ICC Profile Tool</v>
       </c>
       <c r="B117" t="str">
-        <v>(optional)</v>
+        <v>ICC-Profil-Tool</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>e.g. evaluating ICC profiles for press calibration</v>
+        <v>Powered by {lib}</v>
       </c>
       <c r="B118" t="str">
-        <v>z. B. ICC-Profile für Druckkalibrierung evaluieren</v>
+        <v>Betrieben mit {lib}</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>I agree to receive emails about profiletool releases. I can unsubscribe at any time.</v>
+        <v>Subscribe</v>
       </c>
       <c r="B119" t="str">
-        <v>Ich willige ein, E-Mails über profiletool-Releases zu erhalten. Ich kann mich jederzeit abmelden.</v>
+        <v>Abonnieren</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>Cancel</v>
+        <v>Get notified about new profiletool releases</v>
       </c>
       <c r="B120" t="str">
-        <v>Abbrechen</v>
+        <v>Bei neuen profiletool-Releases benachrichtigt werden</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>Subscribe</v>
+        <v>Get notified about new releases</v>
       </c>
       <c r="B121" t="str">
-        <v>Abonnieren</v>
+        <v>Bei neuen Releases benachrichtigt werden</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>Thanks — we’ll be in touch.</v>
+        <v>Close</v>
       </c>
       <c r="B122" t="str">
-        <v>Danke — wir melden uns.</v>
+        <v>Schließen</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>Once approved you’ll receive a welcome email. After that, you’ll only hear from us when a new profiletool release ships.</v>
+        <v>We’ll email you when a new major or minor profiletool release ships. Patch releases are skipped. Your address is reviewed manually before being added.</v>
       </c>
       <c r="B123" t="str">
-        <v>Nach Freigabe erhalten Sie eine Willkommens-E-Mail. Danach hören Sie nur dann von uns, wenn ein neues profiletool-Release erscheint.</v>
+        <v>Wir benachrichtigen Sie per E-Mail, sobald ein neues Major- oder Minor-Release von profiletool erscheint. Patch-Releases werden übersprungen. Ihre Adresse wird manuell geprüft, bevor sie aufgenommen wird.</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>Close</v>
+        <v>Email address</v>
       </c>
       <c r="B124" t="str">
-        <v>Schließen</v>
+        <v>E-Mail-Adresse</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>Privacy notice</v>
+        <v>you@example.com</v>
       </c>
       <c r="B125" t="str">
-        <v>Datenschutzhinweis</v>
+        <v>sie@example.com</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>Please enter a valid email address.</v>
+        <v>How will you use profiletool?</v>
       </c>
       <c r="B126" t="str">
-        <v>Bitte geben Sie eine gültige E-Mail-Adresse ein.</v>
+        <v>Wofür werden Sie profiletool nutzen?</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>Too many requests. Please try again later.</v>
+        <v>(optional)</v>
       </c>
       <c r="B127" t="str">
-        <v>Zu viele Anfragen. Bitte versuchen Sie es später erneut.</v>
+        <v>(optional)</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>Please check the form and try again.</v>
+        <v>e.g. evaluating ICC profiles for press calibration</v>
       </c>
       <c r="B128" t="str">
-        <v>Bitte überprüfen Sie das Formular und versuchen Sie es erneut.</v>
+        <v>z. B. ICC-Profile für Druckkalibrierung evaluieren</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>Could not send your request. Please try again.</v>
+        <v>I agree to receive emails about profiletool releases. I can unsubscribe at any time.</v>
       </c>
       <c r="B129" t="str">
-        <v>Anfrage konnte nicht gesendet werden. Bitte versuchen Sie es erneut.</v>
+        <v>Ich willige ein, E-Mails über profiletool-Releases zu erhalten. Ich kann mich jederzeit abmelden.</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>Network error. Please try again.</v>
+        <v>Cancel</v>
       </c>
       <c r="B130" t="str">
-        <v>Netzwerkfehler. Bitte versuchen Sie es erneut.</v>
+        <v>Abbrechen</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>Error:</v>
+        <v>Subscribe</v>
       </c>
       <c r="B131" t="str">
-        <v>Fehler:</v>
+        <v>Abonnieren</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>Convert to XML</v>
+        <v>Thanks — we’ll be in touch.</v>
       </c>
       <c r="B132" t="str">
-        <v>In XML konvertieren</v>
+        <v>Danke — wir melden uns.</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>Convert to JSON</v>
+        <v>Once approved you’ll receive a welcome email. After that, you’ll only hear from us when a new profiletool release ships.</v>
       </c>
       <c r="B133" t="str">
-        <v>In JSON konvertieren</v>
+        <v>Nach Freigabe erhalten Sie eine Willkommens-E-Mail. Danach hören Sie nur dann von uns, wenn ein neues profiletool-Release erscheint.</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>Convert to ICC</v>
+        <v>Close</v>
       </c>
       <c r="B134" t="str">
-        <v>In ICC konvertieren</v>
+        <v>Schließen</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>Converting to XML…</v>
+        <v>Privacy notice</v>
       </c>
       <c r="B135" t="str">
-        <v>Konvertiere in XML…</v>
+        <v>Datenschutzhinweis</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>Converting to JSON…</v>
+        <v>Please enter a valid email address.</v>
       </c>
       <c r="B136" t="str">
-        <v>Konvertiere in JSON…</v>
+        <v>Bitte geben Sie eine gültige E-Mail-Adresse ein.</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>Converting to ICC…</v>
+        <v>Too many requests. Please try again later.</v>
       </c>
       <c r="B137" t="str">
-        <v>Konvertiere in ICC…</v>
+        <v>Zu viele Anfragen. Bitte versuchen Sie es später erneut.</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>Load ICC profile</v>
+        <v>Please check the form and try again.</v>
       </c>
       <c r="B138" t="str">
-        <v>ICC-Profil laden</v>
+        <v>Bitte überprüfen Sie das Formular und versuchen Sie es erneut.</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>Drop zone for ICC profile files</v>
+        <v>Could not send your request. Please try again.</v>
       </c>
       <c r="B139" t="str">
-        <v>Ablagebereich für ICC-Profil-Dateien</v>
+        <v>Anfrage konnte nicht gesendet werden. Bitte versuchen Sie es erneut.</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>Profile ID</v>
+        <v>Network error. Please try again.</v>
       </c>
       <c r="B140" t="str">
-        <v>Profil-ID</v>
+        <v>Netzwerkfehler. Bitte versuchen Sie es erneut.</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>No tags found.</v>
+        <v>Error:</v>
       </c>
       <c r="B141" t="str">
-        <v>Keine Tags gefunden.</v>
+        <v>Fehler:</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>Tag Name</v>
+        <v>Convert to XML</v>
       </c>
       <c r="B142" t="str">
-        <v>Tag-Name</v>
+        <v>In XML konvertieren</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>ID</v>
+        <v>Convert to JSON</v>
       </c>
       <c r="B143" t="str">
-        <v>ID</v>
+        <v>In JSON konvertieren</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>Offset</v>
+        <v>Convert to ICC</v>
       </c>
       <c r="B144" t="str">
-        <v>Offset</v>
+        <v>In ICC konvertieren</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>Size</v>
+        <v>Converting to XML…</v>
       </c>
       <c r="B145" t="str">
-        <v>Größe</v>
+        <v>Konvertiere in XML…</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>Pad</v>
+        <v>Converting to JSON…</v>
       </c>
       <c r="B146" t="str">
-        <v>Auffüllung</v>
+        <v>Konvertiere in JSON…</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>Bytes changed since load</v>
+        <v>Converting to ICC…</v>
       </c>
       <c r="B147" t="str">
-        <v>Bytes seit dem Laden geändert</v>
+        <v>Konvertiere in ICC…</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>Type</v>
+        <v>Load ICC profile</v>
       </c>
       <c r="B148" t="str">
-        <v>Typ</v>
+        <v>ICC-Profil laden</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>Array of {type}</v>
+        <v>Drop zone for ICC profile files</v>
       </c>
       <c r="B149" t="str">
-        <v>Array von {type}</v>
+        <v>Ablagebereich für ICC-Profil-Dateien</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>(No content)</v>
+        <v>Profile ID</v>
       </c>
       <c r="B150" t="str">
-        <v>(Kein Inhalt)</v>
+        <v>Profil-ID</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>bytes</v>
+        <v>No tags found.</v>
       </c>
       <c r="B151" t="str">
-        <v>Bytes</v>
+        <v>Keine Tags gefunden.</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>Loading full description…</v>
+        <v>Tag Name</v>
       </c>
       <c r="B152" t="str">
-        <v>Lade vollständige Beschreibung…</v>
+        <v>Tag-Name</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>Could not load full description:</v>
+        <v>ID</v>
       </c>
       <c r="B153" t="str">
-        <v>Vollständige Beschreibung konnte nicht geladen werden:</v>
+        <v>ID</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>This profile could not be fully parsed and must not be applied. The header and tag directory below are shown for inspection only.</v>
+        <v>Offset</v>
       </c>
       <c r="B154" t="str">
-        <v>Dieses Profil konnte nicht vollständig gelesen werden und darf nicht angewendet werden. Der Header und das Tag-Verzeichnis unten dienen nur zur Ansicht.</v>
+        <v>Offset</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>Tag contents unavailable — the profile could not be fully parsed.</v>
+        <v>Size</v>
       </c>
       <c r="B155" t="str">
-        <v>Tag-Inhalt nicht verfügbar — das Profil konnte nicht vollständig gelesen werden.</v>
+        <v>Größe</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>No validation output</v>
+        <v>Pad</v>
       </c>
       <c r="B156" t="str">
-        <v>Keine Validierungsausgabe</v>
+        <v>Auffüllung</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>Profile is valid</v>
+        <v>Bytes changed since load</v>
       </c>
       <c r="B157" t="str">
-        <v>Profil ist gültig</v>
+        <v>Bytes seit dem Laden geändert</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>Profile has warning(s)</v>
+        <v>Type</v>
       </c>
       <c r="B158" t="str">
-        <v>Profil hat Warnung(en)</v>
+        <v>Typ</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>Profile is non-compliant</v>
+        <v>Array of {type}</v>
       </c>
       <c r="B159" t="str">
-        <v>Profil ist nicht konform</v>
+        <v>Array von {type}</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>Critical validation error</v>
+        <v>(No content)</v>
       </c>
       <c r="B160" t="str">
-        <v>Kritischer Validierungsfehler</v>
+        <v>(Kein Inhalt)</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>Unknown validation status</v>
+        <v>bytes</v>
       </c>
       <c r="B161" t="str">
-        <v>Unbekannter Validierungsstatus</v>
+        <v>Bytes</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>Critical — shown for inspection only</v>
+        <v>Loading full description…</v>
       </c>
       <c r="B162" t="str">
-        <v>Kritisch — nur zur Ansicht angezeigt</v>
+        <v>Lade vollständige Beschreibung…</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>No warnings or errors found.</v>
+        <v>Could not load full description:</v>
       </c>
       <c r="B163" t="str">
-        <v>Keine Warnungen oder Fehler gefunden.</v>
+        <v>Vollständige Beschreibung konnte nicht geladen werden:</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>Valid</v>
+        <v>This profile could not be fully parsed and must not be applied. The header and tag directory below are shown for inspection only.</v>
       </c>
       <c r="B164" t="str">
-        <v>Gültig</v>
+        <v>Dieses Profil konnte nicht vollständig gelesen werden und darf nicht angewendet werden. Der Header und das Tag-Verzeichnis unten dienen nur zur Ansicht.</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>Warning</v>
+        <v>Tag contents unavailable — the profile could not be fully parsed.</v>
       </c>
       <c r="B165" t="str">
-        <v>Warnung</v>
+        <v>Tag-Inhalt nicht verfügbar — das Profil konnte nicht vollständig gelesen werden.</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>Error</v>
+        <v>No validation output</v>
       </c>
       <c r="B166" t="str">
-        <v>Fehler</v>
+        <v>Keine Validierungsausgabe</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>Unknown</v>
+        <v>Profile is valid</v>
       </c>
       <c r="B167" t="str">
-        <v>Unbekannt</v>
+        <v>Profil ist gültig</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>Pass</v>
+        <v>Profile has warning(s)</v>
       </c>
       <c r="B168" t="str">
-        <v>Bestanden</v>
+        <v>Profil hat Warnung(en)</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>Fail</v>
+        <v>Profile is non-compliant</v>
       </c>
       <c r="B169" t="str">
-        <v>Fehlgeschlagen</v>
+        <v>Profil ist nicht konform</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>View in context</v>
+        <v>Critical validation error</v>
       </c>
       <c r="B170" t="str">
-        <v>Im Kontext anzeigen</v>
+        <v>Kritischer Validierungsfehler</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>Validation detail</v>
+        <v>Unknown validation status</v>
       </c>
       <c r="B171" t="str">
-        <v>Validierungsdetail</v>
+        <v>Unbekannter Validierungsstatus</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>Triggered by</v>
+        <v>Critical — shown for inspection only</v>
       </c>
       <c r="B172" t="str">
-        <v>Ausgelöst durch</v>
+        <v>Kritisch — nur zur Ansicht angezeigt</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>Field</v>
+        <v>No warnings or errors found.</v>
       </c>
       <c r="B173" t="str">
-        <v>Feld</v>
+        <v>Keine Warnungen oder Fehler gefunden.</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>Current value</v>
+        <v>Valid</v>
       </c>
       <c r="B174" t="str">
-        <v>Aktueller Wert</v>
+        <v>Gültig</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>Required: 0</v>
+        <v>Warning</v>
       </c>
       <c r="B175" t="str">
-        <v>Erforderlich: 0</v>
+        <v>Warnung</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>Expected: {value}</v>
+        <v>Error</v>
       </c>
       <c r="B176" t="str">
-        <v>Erwartet: {value}</v>
+        <v>Fehler</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>Invalid</v>
+        <v>Unknown</v>
       </c>
       <c r="B177" t="str">
-        <v>Ungültig</v>
+        <v>Unbekannt</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>This finding couldn't be tied to a specific field.</v>
+        <v>Pass</v>
       </c>
       <c r="B178" t="str">
-        <v>Dieser Befund konnte keinem bestimmten Feld zugeordnet werden.</v>
+        <v>Bestanden</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>Close</v>
+        <v>Fail</v>
       </c>
       <c r="B179" t="str">
-        <v>Schließen</v>
+        <v>Fehlgeschlagen</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>Loading XML editor…</v>
+        <v>View in context</v>
       </c>
       <c r="B180" t="str">
-        <v>Lade XML-Editor…</v>
+        <v>Im Kontext anzeigen</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>Loading JSON editor…</v>
+        <v>Validation detail</v>
       </c>
       <c r="B181" t="str">
-        <v>Lade JSON-Editor…</v>
+        <v>Validierungsdetail</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>You have unsaved XML edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+        <v>Triggered by</v>
       </c>
       <c r="B182" t="str">
-        <v>Sie haben nicht gespeicherte XML-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+        <v>Ausgelöst durch</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>You have unsaved JSON edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+        <v>Field</v>
       </c>
       <c r="B183" t="str">
-        <v>Sie haben nicht gespeicherte JSON-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+        <v>Feld</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>● unsaved XML edits</v>
+        <v>Current value</v>
       </c>
       <c r="B184" t="str">
-        <v>● nicht gespeicherte XML-Änderungen</v>
+        <v>Aktueller Wert</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>● unsaved JSON edits</v>
+        <v>Required: 0</v>
       </c>
       <c r="B185" t="str">
-        <v>● nicht gespeicherte JSON-Änderungen</v>
+        <v>Erforderlich: 0</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>Click &lt;em&gt;Convert to XML&lt;/em&gt; to generate an editable XML representation of this profile. The XML is produced by the same IccLibXML code path used by the upstream &lt;code&gt;IccToXml&lt;/code&gt; tool.</v>
+        <v>Expected: {value}</v>
       </c>
       <c r="B186" t="str">
-        <v>Klicken Sie auf &lt;em&gt;In XML konvertieren&lt;/em&gt;, um eine bearbeitbare XML-Darstellung dieses Profils zu erzeugen. Das XML wird vom gleichen IccLibXML-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToXml&lt;/code&gt; verwendet.</v>
+        <v>Erwartet: {value}</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>Click &lt;em&gt;Convert to JSON&lt;/em&gt; to generate an editable JSON representation of this profile. The JSON is produced by the same IccLibJSON code path used by the upstream &lt;code&gt;IccToJson&lt;/code&gt; tool.</v>
+        <v>Invalid</v>
       </c>
       <c r="B187" t="str">
-        <v>Klicken Sie auf &lt;em&gt;In JSON konvertieren&lt;/em&gt;, um eine bearbeitbare JSON-Darstellung dieses Profils zu erzeugen. Das JSON wird vom gleichen IccLibJSON-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToJson&lt;/code&gt; verwendet.</v>
+        <v>Ungültig</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>indent</v>
+        <v>This finding couldn't be tied to a specific field.</v>
       </c>
       <c r="B188" t="str">
-        <v>Einrückung</v>
+        <v>Dieser Befund konnte keinem bestimmten Feld zugeordnet werden.</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>sort keys</v>
+        <v>Close</v>
       </c>
       <c r="B189" t="str">
-        <v>Schlüssel sortieren</v>
+        <v>Schließen</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
+        <v>Loading XML editor…</v>
+      </c>
+      <c r="B190" t="str">
+        <v>Lade XML-Editor…</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>Loading JSON editor…</v>
+      </c>
+      <c r="B191" t="str">
+        <v>Lade JSON-Editor…</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>You have unsaved XML edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+      </c>
+      <c r="B192" t="str">
+        <v>Sie haben nicht gespeicherte XML-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>You have unsaved JSON edits. Overwrite them with a fresh conversion from the ICC profile?</v>
+      </c>
+      <c r="B193" t="str">
+        <v>Sie haben nicht gespeicherte JSON-Änderungen. Mit einer neuen Konvertierung aus dem ICC-Profil überschreiben?</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>● unsaved XML edits</v>
+      </c>
+      <c r="B194" t="str">
+        <v>● nicht gespeicherte XML-Änderungen</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>● unsaved JSON edits</v>
+      </c>
+      <c r="B195" t="str">
+        <v>● nicht gespeicherte JSON-Änderungen</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>Click &lt;em&gt;Convert to XML&lt;/em&gt; to generate an editable XML representation of this profile. The XML is produced by the same IccLibXML code path used by the upstream &lt;code&gt;IccToXml&lt;/code&gt; tool.</v>
+      </c>
+      <c r="B196" t="str">
+        <v>Klicken Sie auf &lt;em&gt;In XML konvertieren&lt;/em&gt;, um eine bearbeitbare XML-Darstellung dieses Profils zu erzeugen. Das XML wird vom gleichen IccLibXML-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToXml&lt;/code&gt; verwendet.</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>Click &lt;em&gt;Convert to JSON&lt;/em&gt; to generate an editable JSON representation of this profile. The JSON is produced by the same IccLibJSON code path used by the upstream &lt;code&gt;IccToJson&lt;/code&gt; tool.</v>
+      </c>
+      <c r="B197" t="str">
+        <v>Klicken Sie auf &lt;em&gt;In JSON konvertieren&lt;/em&gt;, um eine bearbeitbare JSON-Darstellung dieses Profils zu erzeugen. Das JSON wird vom gleichen IccLibJSON-Codepfad erzeugt, den auch das Upstream-Tool &lt;code&gt;IccToJson&lt;/code&gt; verwendet.</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>indent</v>
+      </c>
+      <c r="B198" t="str">
+        <v>Einrückung</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>sort keys</v>
+      </c>
+      <c r="B199" t="str">
+        <v>Schlüssel sortieren</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
         <v>Profile written from edits, but re-validation failed:</v>
       </c>
-      <c r="B190" t="str">
+      <c r="B200" t="str">
         <v>Profil aus Änderungen geschrieben, aber Neuvalidierung fehlgeschlagen:</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B190"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B200"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>